<commit_message>
Introduce telop notation v2 and validator; migrate ep1 conte
- Notation v2: one telop per line (Sn/本文), S1/全文 keyword,
  《》emphasis marker, structured tags in motion column,
  production notes banned from text column
- Rules written into 第1回 workbook as テロップ記法v2 sheet
- validate_telops.py: flags violations instead of stripping them
- 40 of 55 ep1 cuts rewritten to v2 (zero violations now);
  change log in mg_factory/design_reference
- ep2 workbook still has 33 violations (mostly S1/字幕全文 -> S1/全文);
  left untouched because the file is currently open in Excel

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/第1回_コンテ表_v1.xlsx
+++ b/第1回_コンテ表_v1.xlsx
@@ -12,6 +12,7 @@
     <sheet name="BGM_SUNO" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="SE一覧" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="テロップ規定" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="テロップ記法v2" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'MG制作計画'!$A$1:$M$38</definedName>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="ＭＳ Ｐゴシック"/>
       <family val="2"/>
@@ -81,6 +82,10 @@
       <b val="1"/>
       <color rgb="001A1A1A"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font/>
   </fonts>
   <fills count="13">
     <fill>
@@ -172,7 +177,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -246,6 +251,8 @@
     <xf numFmtId="0" fontId="9" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -1043,12 +1050,16 @@
       </c>
       <c r="P2" s="5" t="inlineStr">
         <is>
-          <t>S6/サムネ文言そのもの(日本、終わる 等)</t>
+          <t>S6/日本、終わる
+S6/年金、消える
+S6/知らないと、損する</t>
         </is>
       </c>
       <c r="Q2" s="5" t="inlineStr">
         <is>
-          <t>1枚ごとにスケール105→100%のドン付き出現 [maxchar:10]</t>
+          <t>1枚ごとにスケール105→100%のドン付き出現 [maxchar:10] [role:in-thumb] #S6はサムネ画像内の文字。詳細はC01_偽サムネ制作仕様_v1.md
+〃
+〃</t>
         </is>
       </c>
       <c r="R2" s="5" t="inlineStr">
@@ -1289,7 +1300,7 @@
       </c>
       <c r="Q4" s="5" t="inlineStr">
         <is>
-          <t>字幕フェードイン。「同じ手口」のみ字間+100に広げる</t>
+          <t>字幕フェードイン [emph:同じ手口|字間+100]</t>
         </is>
       </c>
       <c r="R4" s="5" t="inlineStr">
@@ -1408,12 +1419,14 @@
       </c>
       <c r="P5" s="5" t="inlineStr">
         <is>
-          <t>S1/ぼくは15年、地方のケーブルテレビで、ニュースやドキュメンタリーを撮ってきました+画面隅に小さく「15年」S5</t>
+          <t>S1/ぼくは15年、地方のケーブルテレビで、ニュースやドキュメンタリーを撮ってきました
+S5/15年</t>
         </is>
       </c>
       <c r="Q5" s="16" t="inlineStr">
         <is>
-          <t>字幕フェードイン/「15年」は数字だけ先に出す [pos:right] [offset:300,-380]</t>
+          <t>字幕フェードイン
+数字だけ先に出す [pos:right] [offset:300,-380]</t>
         </is>
       </c>
       <c r="R5" s="5" t="inlineStr">
@@ -1505,7 +1518,7 @@
       </c>
       <c r="Q6" s="5" t="inlineStr">
         <is>
-          <t>字幕フェードイン。「——」で0.5秒の間に合わせ字幕も2段階表示</t>
+          <t>字幕フェードイン [sync:「——」の0.5秒の間で2段階表示]</t>
         </is>
       </c>
       <c r="R6" s="5" t="inlineStr">
@@ -1620,12 +1633,14 @@
       </c>
       <c r="P7" s="5" t="inlineStr">
         <is>
-          <t>S2/狂っている、とすら思いました。(この一文のみ)</t>
+          <t>S2/狂っている、とすら思いました。
+S1/全文</t>
         </is>
       </c>
       <c r="Q7" s="5" t="inlineStr">
         <is>
-          <t>★文:画面が一瞬暗転し中央に1文字ずつ2Fずらしでフェードイン。他の文はS1下部字幕 [pos:bottom]</t>
+          <t>★文:画面が一瞬暗転し中央に1文字ずつ2Fずらしでフェードイン [pos:center]
+下部字幕</t>
         </is>
       </c>
       <c r="R7" s="5" t="inlineStr">
@@ -1832,12 +1847,14 @@
       </c>
       <c r="P9" s="5" t="inlineStr">
         <is>
-          <t>S2/なぜ、こうなってしまったんだろう。(2つの問いを順に中央表示)</t>
+          <t>S2/なぜ、こうなってしまったんだろう。
+S2/なぜ、みんな、数字に取り憑かれてしまうんだろう。</t>
         </is>
       </c>
       <c r="Q9" s="5" t="inlineStr">
         <is>
-          <t>中央・1問ずつフェードイン→アウト。字間広め</t>
+          <t>中央・フェードイン→アウト。字間広め [seq:順次]
+〃</t>
         </is>
       </c>
       <c r="R9" s="5" t="inlineStr">
@@ -1925,7 +1942,7 @@
       </c>
       <c r="P10" s="5" t="inlineStr">
         <is>
-          <t>S2/このチャンネルは、その記録です。(この一文のみ)</t>
+          <t>S2/このチャンネルは、その記録です。</t>
         </is>
       </c>
       <c r="Q10" s="5" t="inlineStr">
@@ -2017,12 +2034,14 @@
       </c>
       <c r="P11" s="5" t="inlineStr">
         <is>
-          <t>S2/ぜんぶ、売り物になっていく(タイトル)+S1字幕でナレ全文</t>
+          <t>S2/ぜんぶ、売り物になっていく
+S1/全文</t>
         </is>
       </c>
       <c r="Q11" s="5" t="inlineStr">
         <is>
-          <t>タイトル:字間が広い状態から通常へ収束しつつフェードイン</t>
+          <t>タイトル:字間が広い状態から通常へ収束しつつフェードイン [role:title]
+下部字幕</t>
         </is>
       </c>
       <c r="R11" s="5" t="inlineStr">
@@ -2142,12 +2161,12 @@
       </c>
       <c r="P12" s="7" t="inlineStr">
         <is>
-          <t>S2/不安は、商品ではありません。エサです。</t>
+          <t>S2/不安は、商品ではありません。《エサです。》</t>
         </is>
       </c>
       <c r="Q12" s="7" t="inlineStr">
         <is>
-          <t>★文:下1/3中央。「エサです。」だけ2F遅れて出現+金茶#C9A063 [pos:bottom]</t>
+          <t>★文:下1/3中央 [pos:bottom] [emph:エサです。|金茶,2F遅れて出現]</t>
         </is>
       </c>
       <c r="R12" s="7" t="inlineStr">
@@ -2234,12 +2253,12 @@
       </c>
       <c r="P13" s="7" t="inlineStr">
         <is>
-          <t>S1/字幕全文。「伸びます」に合わせグラフ内テロップも同期</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q13" s="7" t="inlineStr">
         <is>
-          <t>字幕フェード/グラフラベルはカウントアップ</t>
+          <t>字幕フェード [sync:「伸びます」の語でグラフ内ラベルのカウントアップを同期]</t>
         </is>
       </c>
       <c r="R13" s="7" t="inlineStr">
@@ -2357,12 +2376,12 @@
       </c>
       <c r="P14" s="7" t="inlineStr">
         <is>
-          <t>S2/売られているのは、あなたの「注意」です。</t>
+          <t>S2/売られているのは、あなたの《「注意」》です。</t>
         </is>
       </c>
       <c r="Q14" s="7" t="inlineStr">
         <is>
-          <t>★文:中央。「注意」のみ金茶+鍵括弧を1.2倍</t>
+          <t>★文:中央 [emph:「注意」|金茶,鍵括弧1.2倍]</t>
         </is>
       </c>
       <c r="R14" s="7" t="inlineStr">
@@ -2479,12 +2498,14 @@
       </c>
       <c r="P15" s="7" t="inlineStr">
         <is>
-          <t>S2/感情は、編集で作れます。+デモ内に「同じ映像です」の小テロップS1</t>
+          <t>S2/感情は、編集で作れます。
+S1/同じ映像です</t>
         </is>
       </c>
       <c r="Q15" s="7" t="inlineStr">
         <is>
-          <t>★文:デモ終了直後に中央、静かにフェード</t>
+          <t>★文:デモ終了直後に中央、静かにフェード
+デモ内に小さく表示 [role:in-demo]</t>
         </is>
       </c>
       <c r="R15" s="7" t="inlineStr">
@@ -2598,12 +2619,16 @@
       </c>
       <c r="P16" s="7" t="inlineStr">
         <is>
-          <t>S5/「MIT 2018」「約12万件」を画面主役に。S1字幕併走</t>
+          <t>S5/MIT 2018
+S5/約12万件
+S1/全文</t>
         </is>
       </c>
       <c r="Q16" s="17" t="inlineStr">
         <is>
-          <t>数字カウントアップ+スタンプ着地 [maxchar:12]</t>
+          <t>数字カウントアップ+スタンプ着地 [maxchar:12]
+〃
+下部字幕</t>
         </is>
       </c>
       <c r="R16" s="7" t="inlineStr">
@@ -2723,12 +2748,16 @@
       </c>
       <c r="P17" s="7" t="inlineStr">
         <is>
-          <t>S2/ウソのほうが、速く、遠くまで広がっていました。+線ラベル「ウソ」「本当」S5</t>
+          <t>S2/ウソのほうが、速く、遠くまで広がっていました。
+S5/ウソ
+S5/本当</t>
         </is>
       </c>
       <c r="Q17" s="7" t="inlineStr">
         <is>
-          <t>★文:グラフ下に固定表示のまま4秒保持</t>
+          <t>★文:グラフ下に固定表示のまま4秒保持 [pos:bottom]
+線ラベル(グラフ内) [role:in-graph]
+〃</t>
         </is>
       </c>
       <c r="R17" s="7" t="inlineStr">
@@ -2845,12 +2874,12 @@
       </c>
       <c r="P18" s="7" t="inlineStr">
         <is>
-          <t>S1/字幕全文。「つい」3箇所のみ金茶</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q18" s="7" t="inlineStr">
         <is>
-          <t>字幕フェード。「つい」は出現を2Fずつ遅らせ律動を作る</t>
+          <t>字幕フェード [emph:つい|金茶,3箇所を2Fずつ遅らせ律動]</t>
         </is>
       </c>
       <c r="R18" s="7" t="inlineStr">
@@ -3081,7 +3110,7 @@
       </c>
       <c r="P20" s="7" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q20" s="7" t="inlineStr">
@@ -3323,7 +3352,7 @@
       </c>
       <c r="P22" s="7" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q22" s="7" t="inlineStr">
@@ -3443,12 +3472,14 @@
       </c>
       <c r="P23" s="9" t="inlineStr">
         <is>
-          <t>S1/字幕全文+画面隅に小さく「1920s NEW YORK」S5(欧文)</t>
+          <t>S1/全文
+S5(欧文)/1920s NEW YORK</t>
         </is>
       </c>
       <c r="Q23" s="18" t="inlineStr">
         <is>
-          <t>字幕フェード/年代表記はタイプ風に [pos:right] [offset:300,-380]</t>
+          <t>字幕フェード
+タイプ風に出現 [pos:right] [offset:300,-380]</t>
         </is>
       </c>
       <c r="R23" s="9" t="inlineStr">
@@ -3536,7 +3567,7 @@
       </c>
       <c r="P24" s="9" t="inlineStr">
         <is>
-          <t>S3/「女性にも、たばこを吸わせたい」。(引用スタイル)</t>
+          <t>S3/「女性にも、たばこを吸わせたい」。</t>
         </is>
       </c>
       <c r="Q24" s="9" t="inlineStr">
@@ -3846,12 +3877,12 @@
       </c>
       <c r="P27" s="9" t="inlineStr">
         <is>
-          <t>S1/字幕全文。「まったく同じ文法です」のみ金茶</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q27" s="9" t="inlineStr">
         <is>
-          <t>字幕フェード</t>
+          <t>字幕フェード [emph:まったく同じ文法です|金茶]</t>
         </is>
       </c>
       <c r="R27" s="9" t="inlineStr">
@@ -3968,12 +3999,14 @@
       </c>
       <c r="P28" s="9" t="inlineStr">
         <is>
-          <t>S5(欧文)/PROPAGANDA(表紙合成)+S1字幕</t>
+          <t>S5(欧文)/PROPAGANDA
+S1/全文</t>
         </is>
       </c>
       <c r="Q28" s="9" t="inlineStr">
         <is>
-          <t>タイトル:型押しが光でなぞられるモーション</t>
+          <t>表紙に合成。型押しが光でなぞられる [role:in-image]
+下部字幕</t>
         </is>
       </c>
       <c r="R28" s="9" t="inlineStr">
@@ -4086,7 +4119,7 @@
       </c>
       <c r="P29" s="9" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q29" s="9" t="inlineStr">
@@ -4272,12 +4305,16 @@
       </c>
       <c r="P31" s="9" t="inlineStr">
         <is>
-          <t>S2/複雑なことを、単純な対立にする。/敵を、名指しする。/何度も繰り返す。(3行順次)</t>
+          <t>S2/複雑なことを、単純な対立にする。
+S2/敵を、名指しする。
+S2/何度も繰り返す。</t>
         </is>
       </c>
       <c r="Q31" s="9" t="inlineStr">
         <is>
-          <t>3行が上から順にスタンプ的に出現(各1拍)</t>
+          <t>3行が上から順にスタンプ的に出現(各1拍) [seq:順次]
+〃
+〃</t>
         </is>
       </c>
       <c r="R31" s="9" t="inlineStr">
@@ -4513,7 +4550,7 @@
       </c>
       <c r="P33" s="9" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q33" s="9" t="inlineStr">
@@ -4724,12 +4761,16 @@
       </c>
       <c r="P35" s="9" t="inlineStr">
         <is>
-          <t>S5/「2016」「何千万人分」を画面内で強調+S1字幕</t>
+          <t>S5/2016
+S5/何千万人分
+S1/全文</t>
         </is>
       </c>
       <c r="Q35" s="18" t="inlineStr">
         <is>
-          <t>数字スタンプ+字幕フェード [maxchar:12]</t>
+          <t>数字スタンプ [maxchar:12]
+〃
+下部字幕</t>
         </is>
       </c>
       <c r="R35" s="9" t="inlineStr">
@@ -4842,12 +4883,12 @@
       </c>
       <c r="P36" s="9" t="inlineStr">
         <is>
-          <t>S1/字幕全文。「不安」「怒り」のみ左右の画面色と同色</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q36" s="9" t="inlineStr">
         <is>
-          <t>字幕フェード+2語のみ色同期</t>
+          <t>字幕フェード [emph:不安|左画面と同色] [emph:怒り|右画面と同色]</t>
         </is>
       </c>
       <c r="R36" s="9" t="inlineStr">
@@ -4960,12 +5001,14 @@
       </c>
       <c r="P37" s="9" t="inlineStr">
         <is>
-          <t>S2/その手口が実際に使われたことは、事実です。+S5「2018」</t>
+          <t>S2/その手口が実際に使われたことは、事実です。
+S5/2018</t>
         </is>
       </c>
       <c r="Q37" s="9" t="inlineStr">
         <is>
-          <t>★文:紙面の上に静かに固定表示</t>
+          <t>★文:紙面の上に静かに固定表示
+数字スタンプ [role:in-image]</t>
         </is>
       </c>
       <c r="R37" s="9" t="inlineStr">
@@ -5080,12 +5123,12 @@
       </c>
       <c r="P38" s="9" t="inlineStr">
         <is>
-          <t>S1/字幕全文のみ(装飾一切なし)。★文もS1のまま(この区間だけ強調を封印)</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q38" s="9" t="inlineStr">
         <is>
-          <t>字幕フェードのみ</t>
+          <t>字幕フェードのみ #この区間だけ強調を封印(★文もS1のまま・装飾一切なし)</t>
         </is>
       </c>
       <c r="R38" s="9" t="inlineStr">
@@ -5294,7 +5337,7 @@
       </c>
       <c r="P40" s="11" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q40" s="11" t="inlineStr">
@@ -5387,12 +5430,12 @@
       </c>
       <c r="P41" s="11" t="inlineStr">
         <is>
-          <t>S4/友達は、お金で買えます。(C20と同一スタイル・同一位置)</t>
+          <t>S4/友達は、お金で買えます。</t>
         </is>
       </c>
       <c r="Q41" s="11" t="inlineStr">
         <is>
-          <t>C20と同一モーション(同一性が演出)</t>
+          <t>C20と同一モーション・同一位置(同一性が演出)</t>
         </is>
       </c>
       <c r="R41" s="11" t="inlineStr">
@@ -5510,7 +5553,7 @@
       </c>
       <c r="P42" s="11" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q42" s="11" t="inlineStr">
@@ -5727,12 +5770,14 @@
       </c>
       <c r="P44" s="11" t="inlineStr">
         <is>
-          <t>S5/スマイル ¥0(メニュー内)+S2/人の感情が、商品として提示されている。</t>
+          <t>S5/スマイル ¥0
+S2/人の感情が、商品として提示されている。</t>
         </is>
       </c>
       <c r="Q44" s="19" t="inlineStr">
         <is>
-          <t>メニュー:実在の券売機的な無機質さで。★文:静かに中央下 [pos:bottom]</t>
+          <t>メニュー内に表示。実在の券売機的な無機質さ [role:in-image]
+★文:静かに中央下 [pos:bottom]</t>
         </is>
       </c>
       <c r="R44" s="11" t="inlineStr">
@@ -5845,12 +5890,12 @@
       </c>
       <c r="P45" s="11" t="inlineStr">
         <is>
-          <t>S1/字幕全文。「市場価値」のみ鍵括弧を大きく</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q45" s="11" t="inlineStr">
         <is>
-          <t>字幕フェード</t>
+          <t>字幕フェード [emph:「市場価値」|鍵括弧大きく]</t>
         </is>
       </c>
       <c r="R45" s="11" t="inlineStr">
@@ -6089,12 +6134,12 @@
       </c>
       <c r="P47" s="11" t="inlineStr">
         <is>
-          <t>S2/ぜんぶ、売り物になっていくんです。(タイトル呼応)</t>
+          <t>S2/ぜんぶ、売り物になっていくんです。</t>
         </is>
       </c>
       <c r="Q47" s="11" t="inlineStr">
         <is>
-          <t>★文:値札が消える直前に中央表示→値札と一緒に消える</t>
+          <t>★文:値札が消える直前に中央表示→値札と一緒に消える #タイトル呼応</t>
         </is>
       </c>
       <c r="R47" s="11" t="inlineStr">
@@ -6213,7 +6258,7 @@
       </c>
       <c r="P48" s="13" t="inlineStr">
         <is>
-          <t>S1/字幕全文</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q48" s="13" t="inlineStr">
@@ -6307,12 +6352,16 @@
       </c>
       <c r="P49" s="13" t="inlineStr">
         <is>
-          <t>S2/三行(ひとつ。/ふたつ。/みっつ。)を画面左に縦積み</t>
+          <t>S2/ひとつ。本当は売り物じゃないものまで、どんどん売り物になっています。
+S2/ふたつ。その仕組みは、ぼくたちの「つい反応してしまう」心を、よく知って使ってきます。
+S2/みっつ。——でも、仕組みは、知れば、距離が取れます。</t>
         </is>
       </c>
       <c r="Q49" s="13" t="inlineStr">
         <is>
-          <t>1項ずつフェードイン、既出項は少し暗く残す</t>
+          <t>画面左に縦積み。1項ずつフェードイン、既出項は少し暗く残す [pos:left] [seq:順次]
+〃
+〃</t>
         </is>
       </c>
       <c r="R49" s="13" t="inlineStr">
@@ -6430,12 +6479,12 @@
       </c>
       <c r="P50" s="13" t="inlineStr">
         <is>
-          <t>S1/字幕全文。「怖かったんです」のみわずかに大きく(+4px)</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q50" s="13" t="inlineStr">
         <is>
-          <t>字幕フェード</t>
+          <t>字幕フェード [emph:怖かったんです|size+4px]</t>
         </is>
       </c>
       <c r="R50" s="13" t="inlineStr">
@@ -6617,12 +6666,14 @@
       </c>
       <c r="P52" s="13" t="inlineStr">
         <is>
-          <t>S2/たぶん、その感覚のほうが、正しい。</t>
+          <t>S2/たぶん、その感覚のほうが、正しい。
+S1/全文</t>
         </is>
       </c>
       <c r="Q52" s="13" t="inlineStr">
         <is>
-          <t>★文:中央、4秒保持。他はS1字幕</t>
+          <t>★文:中央、4秒保持
+下部字幕</t>
         </is>
       </c>
       <c r="R52" s="13" t="inlineStr">
@@ -6709,12 +6760,14 @@
       </c>
       <c r="P53" s="15" t="inlineStr">
         <is>
-          <t>S2/『なんだろう』解体(ロゴ扱い)+S1字幕</t>
+          <t>S2/『なんだろう』解体
+S1/全文</t>
         </is>
       </c>
       <c r="Q53" s="15" t="inlineStr">
         <is>
-          <t>ロゴ:線画の分解図が組み上がってから文字がフェード</t>
+          <t>ロゴ:線画の分解図が組み上がってから文字がフェード [role:logo]
+下部字幕</t>
         </is>
       </c>
       <c r="R53" s="15" t="inlineStr">
@@ -6831,12 +6884,12 @@
       </c>
       <c r="P54" s="15" t="inlineStr">
         <is>
-          <t>S1/字幕全文。「線引きごと、公開します」のみ金茶</t>
+          <t>S1/全文</t>
         </is>
       </c>
       <c r="Q54" s="15" t="inlineStr">
         <is>
-          <t>字幕フェード</t>
+          <t>字幕フェード [emph:線引きごと、公開します|金茶]</t>
         </is>
       </c>
       <c r="R54" s="15" t="inlineStr">
@@ -6951,12 +7004,12 @@
       </c>
       <c r="P55" s="15" t="inlineStr">
         <is>
-          <t>S4/あなたの怒りは、誰の収益になっているのか(次回タイトル)</t>
+          <t>S4/あなたの怒りは、誰の収益になっているのか</t>
         </is>
       </c>
       <c r="Q55" s="15" t="inlineStr">
         <is>
-          <t>黒地中央、静かにフェード、3秒保持</t>
+          <t>黒地中央、静かにフェード、3秒保持 [role:next-title]</t>
         </is>
       </c>
       <c r="R55" s="15" t="inlineStr">
@@ -7073,12 +7126,12 @@
       </c>
       <c r="P56" s="15" t="inlineStr">
         <is>
-          <t>S5(欧文)/Score: Unsaid Works→ロゴ</t>
+          <t>S5(欧文)/Score: Unsaid Works</t>
         </is>
       </c>
       <c r="Q56" s="15" t="inlineStr">
         <is>
-          <t>順次フェード(日本語の問いで始まり英語レーベル名で終わる設計)</t>
+          <t>順次フェード→レーベルロゴ(画像)へ #日本語の問いで始まり英語レーベル名で終わる設計</t>
         </is>
       </c>
       <c r="R56" s="15" t="inlineStr">
@@ -10775,4 +10828,266 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>テロップ記法 v2(2026-07-13制定)</t>
+        </is>
+      </c>
+      <c r="B1" s="22" t="inlineStr"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="26" t="inlineStr"/>
+      <c r="B2" s="22" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="25" t="inlineStr">
+        <is>
+          <t>■ テロップ列(スタイル/内容)のルール</t>
+        </is>
+      </c>
+      <c r="B3" s="22" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B4" s="22" t="inlineStr">
+        <is>
+          <t>1行 = 1テロップ。書式は「Sn/本文」(nは1〜6)。欧文は「Sn(欧文)/本文」</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="26" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B5" s="22" t="inlineStr">
+        <is>
+          <t>本文には画面に出す文字だけを書く。制作指示・位置・演出メモは書かない(モーション列へ)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>特殊値「S1/全文」= ナレーション列の全文を字幕にする(旧「字幕全文」)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>強調語は本文中で《》で括る。例: S2/不安は、商品ではありません。《エサです。》 デフォルトの強調=金茶</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="26" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>複数テロップは改行して並べる。順次表示もスタイルを行ごとに繰り返す</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="B9" s="22" t="inlineStr">
+        <is>
+          <t>禁止: 「+」での連結 / (括弧)での指示 / 「〜のみ金茶」「併走」「画面主役」等の指示文の混入</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="26" t="inlineStr"/>
+      <c r="B10" s="22" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="25" t="inlineStr">
+        <is>
+          <t>■ モーション列のルール</t>
+        </is>
+      </c>
+      <c r="B11" s="22" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>テロップ列の行と同順で1行ずつ対応させる。同じ内容の繰り返しは「〃」</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="26" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>構造化タグ: [pos:位置] [offset:x,y] [maxchar:n] [sync:同期先] [seq:順次] [role:役割] [emph:語|効果]</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="26" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B14" s="22" t="inlineStr">
+        <is>
+          <t>[emph:語|効果] は金茶以外の強調(色同期・サイズ変更・字間など)を指定する</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="26" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>[role:] の値: title / logo / next-title / in-thumb / in-image / in-graph / in-demo(画面内合成systemを示す)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="26" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="B16" s="22" t="inlineStr">
+        <is>
+          <t>「#」以降は自由メモ(機械処理の対象外)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="26" t="inlineStr"/>
+      <c r="B17" s="22" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="25" t="inlineStr">
+        <is>
+          <t>■ スタイル別の管理先</t>
+        </is>
+      </c>
+      <c r="B18" s="22" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="26" t="inlineStr">
+        <is>
+          <t>S1</t>
+        </is>
+      </c>
+      <c r="B19" s="22" t="inlineStr">
+        <is>
+          <t>標準字幕。Premiere SRT(conte2srt.py)で管理。Remotionオーバーレイの対象外</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="26" t="inlineStr">
+        <is>
+          <t>S2/S3/S5</t>
+        </is>
+      </c>
+      <c r="B20" s="22" t="inlineStr">
+        <is>
+          <t>RemotionのTelopOverlayで生成(透過mov)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="26" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+      <c r="B21" s="22" t="inlineStr">
+        <is>
+          <t>黒画面宣言はオーバーレイではなくフルフレームカット。JsonScenesのstatement型で作る</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="26" t="inlineStr">
+        <is>
+          <t>S6</t>
+        </is>
+      </c>
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>サムネ画像内の文字。Canva/Photoshop側で制作(オーバーレイ対象外)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="26" t="inlineStr"/>
+      <c r="B23" s="22" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="25" t="inlineStr">
+        <is>
+          <t>■ 検証</t>
+        </is>
+      </c>
+      <c r="B24" s="22" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="26" t="inlineStr"/>
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>python3 validate_telops.py &lt;コンテ表.xlsx&gt; で違反を検出。警告ゼロにしてから変換に進む</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Rebuild TelopOverlay on notation v2 with show design
- conte2telops.py: strict v2 parser conte -> telop JSON (S2/S3/S5 only;
  S1=SRT, S4=statement scenes, S6=in-image, [role:*]=in-MG excluded;
  《》emphasis extraction, pos/offset/maxchar/seq tags)
- TelopOverlay: theme-connected S2 (per-char 2F stagger, gold emphasis),
  S3 quote (slow fade), S5 Oswald (stamp/typewriter); stack groups as
  flex column with dimming; replace-mode sequential; part-window
  rendering (P0-P5) with per-part npm scripts; backdrop prop for
  style-sample stills
- Verified: 6 style samples + transparent ProRes sample (yuva444p12le)
- Add [role:] tags to ep1 conte C13/C15/C55 (rendered inside MG/AE)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/第1回_コンテ表_v1.xlsx
+++ b/第1回_コンテ表_v1.xlsx
@@ -2381,7 +2381,7 @@
       </c>
       <c r="Q14" s="7" t="inlineStr">
         <is>
-          <t>★文:中央 [emph:「注意」|金茶,鍵括弧1.2倍]</t>
+          <t>★文はMG(C13AttentionFlow)内で表示 [role:in-graph] [emph:「注意」|金茶,鍵括弧1.2倍]</t>
         </is>
       </c>
       <c r="R14" s="7" t="inlineStr">
@@ -2626,7 +2626,7 @@
       </c>
       <c r="Q16" s="17" t="inlineStr">
         <is>
-          <t>数字カウントアップ+スタンプ着地 [maxchar:12]
+          <t>数字カウントアップ+スタンプ着地 [maxchar:12] [role:in-graph]
 〃
 下部字幕</t>
         </is>
@@ -7131,7 +7131,7 @@
       </c>
       <c r="Q56" s="15" t="inlineStr">
         <is>
-          <t>順次フェード→レーベルロゴ(画像)へ #日本語の問いで始まり英語レーベル名で終わる設計</t>
+          <t>順次フェード→レーベルロゴ(画像)へ [role:in-image] #エンドカードAEマスター内。日本語の問いで始まり英語レーベル名で終わる設計</t>
         </is>
       </c>
       <c r="R56" s="15" t="inlineStr">

</xml_diff>

<commit_message>
Fix line breaking, orphan cues, and expand keyword emphasis
- conte2srt: v2「全文」support; balanced natural splitting (48 chars =
  2x24 lines), no orphan cues (short tails merge into previous);
  output names derived from input (第1回 -> ep01) to prevent mislabeling
- TelopOverlay: one-line preference with font step-down, balanced
  breaks at 。>、>particle, no orphan lines; emphasis colors (gold 《》 /
  vermilion via [emph:語|朱]) with 12F delayed rise-in beat
- Conte: 26 emphasis marks added across ep1/ep2 (18 of 32 ep1 overlay
  telops now accented; red reserved for 狂っている/ウソ/わざと)
- AGENTS.md: line-break and emphasis rules codified

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/第1回_コンテ表_v1.xlsx
+++ b/第1回_コンテ表_v1.xlsx
@@ -1639,7 +1639,7 @@
       </c>
       <c r="Q7" s="5" t="inlineStr">
         <is>
-          <t>★文:画面が一瞬暗転し中央に1文字ずつ2Fずらしでフェードイン [pos:center]
+          <t>★文:画面が一瞬暗転し中央に1文字ずつ2Fずらしでフェードイン [pos:center] [emph:狂っている、|朱]
 下部字幕</t>
         </is>
       </c>
@@ -1848,7 +1848,7 @@
       <c r="P9" s="5" t="inlineStr">
         <is>
           <t>S2/なぜ、こうなってしまったんだろう。
-S2/なぜ、みんな、数字に取り憑かれてしまうんだろう。</t>
+S2/なぜ、みんな、《数字》に取り憑かれてしまうんだろう。</t>
         </is>
       </c>
       <c r="Q9" s="5" t="inlineStr">
@@ -1942,7 +1942,7 @@
       </c>
       <c r="P10" s="5" t="inlineStr">
         <is>
-          <t>S2/このチャンネルは、その記録です。</t>
+          <t>S2/このチャンネルは、その《記録》です。</t>
         </is>
       </c>
       <c r="Q10" s="5" t="inlineStr">
@@ -2498,7 +2498,7 @@
       </c>
       <c r="P15" s="7" t="inlineStr">
         <is>
-          <t>S2/感情は、編集で作れます。
+          <t>S2/感情は、《編集》で作れます。
 S1/同じ映像です</t>
         </is>
       </c>
@@ -2755,7 +2755,7 @@
       </c>
       <c r="Q17" s="7" t="inlineStr">
         <is>
-          <t>★文:グラフ下に固定表示のまま4秒保持 [pos:bottom]
+          <t>★文:グラフ下に固定表示のまま4秒保持 [pos:bottom] [emph:ウソ|朱]
 線ラベル(グラフ内) [role:in-graph]
 〃</t>
         </is>
@@ -2992,7 +2992,7 @@
       </c>
       <c r="P19" s="7" t="inlineStr">
         <is>
-          <t>S2/あなたの弱さではありません。人間の、仕様です。</t>
+          <t>S2/あなたの弱さではありません。人間の、《仕様》です。</t>
         </is>
       </c>
       <c r="Q19" s="7" t="inlineStr">
@@ -4431,7 +4431,7 @@
       </c>
       <c r="P32" s="9" t="inlineStr">
         <is>
-          <t>S2/変わったのは、「届け方」です。</t>
+          <t>S2/変わったのは、《「届け方」》です。</t>
         </is>
       </c>
       <c r="Q32" s="9" t="inlineStr">
@@ -4643,7 +4643,7 @@
       </c>
       <c r="P34" s="9" t="inlineStr">
         <is>
-          <t>S2/あなた専用に調整して、届けてくる。</t>
+          <t>S2/《あなた専用》に調整して、届けてくる。</t>
         </is>
       </c>
       <c r="Q34" s="9" t="inlineStr">
@@ -5001,7 +5001,7 @@
       </c>
       <c r="P37" s="9" t="inlineStr">
         <is>
-          <t>S2/その手口が実際に使われたことは、事実です。
+          <t>S2/その手口が実際に使われたことは、《事実》です。
 S5/2018</t>
         </is>
       </c>
@@ -5645,7 +5645,7 @@
       </c>
       <c r="P43" s="11" t="inlineStr">
         <is>
-          <t>S2/笑顔にも、値段がついたことがあります。</t>
+          <t>S2/笑顔にも、《値段》がついたことがあります。</t>
         </is>
       </c>
       <c r="Q43" s="11" t="inlineStr">
@@ -5771,7 +5771,7 @@
       <c r="P44" s="11" t="inlineStr">
         <is>
           <t>S5/スマイル ¥0
-S2/人の感情が、商品として提示されている。</t>
+S2/人の感情が、《商品》として提示されている。</t>
         </is>
       </c>
       <c r="Q44" s="19" t="inlineStr">
@@ -6008,7 +6008,7 @@
       </c>
       <c r="P46" s="11" t="inlineStr">
         <is>
-          <t>S2/人間に、市場価値。</t>
+          <t>S2/人間に、《市場価値》。</t>
         </is>
       </c>
       <c r="Q46" s="11" t="inlineStr">
@@ -6134,7 +6134,7 @@
       </c>
       <c r="P47" s="11" t="inlineStr">
         <is>
-          <t>S2/ぜんぶ、売り物になっていくんです。</t>
+          <t>S2/ぜんぶ、《売り物》になっていくんです。</t>
         </is>
       </c>
       <c r="Q47" s="11" t="inlineStr">
@@ -6353,8 +6353,8 @@
       <c r="P49" s="13" t="inlineStr">
         <is>
           <t>S2/ひとつ。本当は売り物じゃないものまで、どんどん売り物になっています。
-S2/ふたつ。その仕組みは、ぼくたちの「つい反応してしまう」心を、よく知って使ってきます。
-S2/みっつ。——でも、仕組みは、知れば、距離が取れます。</t>
+S2/ふたつ。その仕組みは、ぼくたちの《「つい反応してしまう」》心を、よく知って使ってきます。
+S2/みっつ。——でも、仕組みは、知れば、《距離》が取れます。</t>
         </is>
       </c>
       <c r="Q49" s="13" t="inlineStr">
@@ -6571,7 +6571,7 @@
       </c>
       <c r="P51" s="13" t="inlineStr">
         <is>
-          <t>S2/怖がらなくて済むように、することです。</t>
+          <t>S2/《怖がらなくて済む》ように、することです。</t>
         </is>
       </c>
       <c r="Q51" s="13" t="inlineStr">
@@ -6666,7 +6666,7 @@
       </c>
       <c r="P52" s="13" t="inlineStr">
         <is>
-          <t>S2/たぶん、その感覚のほうが、正しい。
+          <t>S2/たぶん、その感覚のほうが、《正しい》。
 S1/全文</t>
         </is>
       </c>

</xml_diff>